<commit_message>
Changed grandma network address to proper vlan
</commit_message>
<xml_diff>
--- a/network.xlsx
+++ b/network.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10920"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/donert/Documents/UACTech/uacdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA6F2A03-1762-7B48-B166-3B9F9BEEF6C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B991B130-1945-D540-B664-D9DA1E4A71C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="3500" windowWidth="30240" windowHeight="16140" xr2:uid="{C276EF8E-8567-464E-98DC-2A8DA10DDBB6}"/>
   </bookViews>
@@ -22,7 +22,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">network!$A$1:$K$38</definedName>
     <definedName name="taxrate">'[1]mixer costs'!$I$2</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -1580,9 +1580,6 @@
     <t>E8CF83FF3955</t>
   </si>
   <si>
-    <t>192.168.0.81</t>
-  </si>
-  <si>
     <t>LAN1</t>
   </si>
   <si>
@@ -1620,6 +1617,9 @@
   </si>
   <si>
     <t>May be come unused if power control is implemented via IP Relay</t>
+  </si>
+  <si>
+    <t>192.168.205.10</t>
   </si>
 </sst>
 </file>
@@ -1915,7 +1915,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -2005,12 +2005,6 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="6" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -4343,7 +4337,7 @@
         <v>34</v>
       </c>
       <c r="E62" s="1" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="F62" s="6"/>
       <c r="G62" s="19"/>
@@ -5377,7 +5371,7 @@
         <v>232</v>
       </c>
       <c r="B100" s="5" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="C100" s="26"/>
       <c r="D100" s="54" t="s">
@@ -6422,19 +6416,19 @@
     </row>
     <row r="142" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A142" s="55" t="s">
+        <v>496</v>
+      </c>
+      <c r="B142" s="5" t="s">
+        <v>494</v>
+      </c>
+      <c r="C142" s="5" t="s">
         <v>497</v>
-      </c>
-      <c r="B142" s="5" t="s">
-        <v>495</v>
-      </c>
-      <c r="C142" s="5" t="s">
-        <v>498</v>
       </c>
       <c r="D142" s="6" t="s">
         <v>486</v>
       </c>
       <c r="E142" s="6" t="s">
-        <v>494</v>
+        <v>507</v>
       </c>
       <c r="F142" s="6"/>
       <c r="G142" s="19" t="s">
@@ -6451,13 +6445,13 @@
     </row>
     <row r="143" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A143" s="55" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="B143" s="5" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="C143" s="5" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="D143" s="6" t="s">
         <v>387</v>
@@ -6470,51 +6464,51 @@
       </c>
       <c r="I143" s="9"/>
       <c r="J143" s="6" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="K143" s="41"/>
     </row>
     <row r="144" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A144" s="59" t="s">
-        <v>503</v>
-      </c>
-      <c r="B144" s="59" t="s">
+      <c r="A144" s="5" t="s">
+        <v>502</v>
+      </c>
+      <c r="B144" s="5" t="s">
         <v>380</v>
       </c>
-      <c r="C144" s="59" t="s">
+      <c r="C144" s="5" t="s">
+        <v>504</v>
+      </c>
+      <c r="D144" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="E144" s="6" t="s">
         <v>505</v>
       </c>
-      <c r="D144" s="60" t="s">
-        <v>34</v>
-      </c>
-      <c r="E144" s="60" t="s">
-        <v>506</v>
-      </c>
-      <c r="F144" s="60"/>
+      <c r="F144" s="6"/>
       <c r="G144" s="19"/>
       <c r="H144" s="18" t="s">
         <v>166</v>
       </c>
-      <c r="I144" s="61"/>
-      <c r="J144" s="60" t="s">
-        <v>504</v>
-      </c>
-      <c r="K144" s="62" t="s">
-        <v>507</v>
+      <c r="I144" s="9"/>
+      <c r="J144" s="6" t="s">
+        <v>503</v>
+      </c>
+      <c r="K144" s="41" t="s">
+        <v>506</v>
       </c>
     </row>
     <row r="145" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A145" s="59"/>
-      <c r="B145" s="59"/>
-      <c r="C145" s="59"/>
-      <c r="D145" s="60"/>
-      <c r="E145" s="60"/>
-      <c r="F145" s="60"/>
+      <c r="A145" s="5"/>
+      <c r="B145" s="5"/>
+      <c r="C145" s="5"/>
+      <c r="D145" s="6"/>
+      <c r="E145" s="6"/>
+      <c r="F145" s="6"/>
       <c r="G145" s="19"/>
       <c r="H145" s="18"/>
-      <c r="I145" s="61"/>
-      <c r="J145" s="60"/>
-      <c r="K145" s="62"/>
+      <c r="I145" s="9"/>
+      <c r="J145" s="6"/>
+      <c r="K145" s="41"/>
     </row>
     <row r="146" spans="1:11" x14ac:dyDescent="0.2">
       <c r="H146"/>

</xml_diff>